<commit_message>
Add mechanic commissions, fuel type, order type, arrival condition, reception photos, and UX improvements
- Commission system: CommissionType enum, commission fields on User entity, WorkOrderMechanic
  table for assigning multiple mechanics per order with configurable commissions
- Fuel type field on vehicles (Gasolina, Diésel, Eléctrico, Híbrido)
- Order type field (Servicio Nuevo, Correctivo, Preventivo, Garantía, Diagnóstico, Revisión)
- Arrival condition field (Rodando, Grúa, Encendido/No rueda, No enciende, Empujado)
- Reception photos in work order form (camera + gallery, max 6)
- Remove initial diagnosis field from work order form
- Delete confirmation dialogs for vehicles (shows plate) and customers (shows name/ID)
- Vehicles sorted by creation date descending
- DB migration v2->v7 with all new fields, tables, and indexes
- Backup/restore updated for all new entities and fields

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Catalogos.xlsx
+++ b/data/Catalogos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\autom\StudioProjects\servielecarandroid\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rolan\AndroidStudioProjects\Serviaux\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8694174-10C4-4EF2-AFF7-101E01F30650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38B21B18-45C6-48A9-A15A-D368C42949CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usuarios" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="258">
   <si>
     <t>Categoria</t>
   </si>
@@ -258,327 +258,60 @@
     <t>Tipo</t>
   </si>
   <si>
-    <t>Sedan</t>
-  </si>
-  <si>
     <t>SUV</t>
   </si>
   <si>
-    <t>Camioneta</t>
-  </si>
-  <si>
-    <t>Jeep</t>
-  </si>
-  <si>
-    <t>4x4</t>
-  </si>
-  <si>
-    <t>Camion</t>
-  </si>
-  <si>
-    <t>Hibrido</t>
-  </si>
-  <si>
-    <t>Electrico</t>
-  </si>
-  <si>
-    <t>Cupe</t>
-  </si>
-  <si>
     <t>VAN</t>
   </si>
   <si>
-    <t>Doble Cabina</t>
-  </si>
-  <si>
     <t>Color</t>
   </si>
   <si>
-    <t>Rojo</t>
-  </si>
-  <si>
-    <t>Azul</t>
-  </si>
-  <si>
-    <t>Amarillo</t>
-  </si>
-  <si>
-    <t>Verde</t>
-  </si>
-  <si>
-    <t>Naranja</t>
-  </si>
-  <si>
-    <t>Morado</t>
-  </si>
-  <si>
-    <t>Rosa</t>
-  </si>
-  <si>
-    <t>Marron</t>
-  </si>
-  <si>
-    <t>Blanco</t>
-  </si>
-  <si>
-    <t>Negro</t>
-  </si>
-  <si>
-    <t>Gris</t>
-  </si>
-  <si>
-    <t>Beige</t>
-  </si>
-  <si>
-    <t>Crema</t>
-  </si>
-  <si>
-    <t>Marfil</t>
-  </si>
-  <si>
-    <t>Celeste</t>
-  </si>
-  <si>
-    <t>Azul Oscuro</t>
-  </si>
-  <si>
-    <t>Verde Claro</t>
-  </si>
-  <si>
-    <t>Verde Oscuro</t>
-  </si>
-  <si>
-    <t>Turquesa</t>
-  </si>
-  <si>
-    <t>Cian</t>
-  </si>
-  <si>
-    <t>Magenta</t>
-  </si>
-  <si>
-    <t>Violeta</t>
-  </si>
-  <si>
-    <t>Dorado</t>
-  </si>
-  <si>
-    <t>Plateado</t>
-  </si>
-  <si>
-    <t>Azul Marino</t>
-  </si>
-  <si>
-    <t>Lima</t>
-  </si>
-  <si>
-    <t>Oliva</t>
-  </si>
-  <si>
-    <t>Plomo</t>
-  </si>
-  <si>
-    <t>Vino</t>
-  </si>
-  <si>
-    <t>Bronce</t>
-  </si>
-  <si>
-    <t>Perla</t>
-  </si>
-  <si>
-    <t>Champagne</t>
-  </si>
-  <si>
     <t>Accesorio</t>
   </si>
   <si>
-    <t>Herramientas Varias</t>
-  </si>
-  <si>
-    <t>Gata</t>
-  </si>
-  <si>
-    <t>Triangulo de Seguridad</t>
-  </si>
-  <si>
-    <t>Botiquin</t>
-  </si>
-  <si>
-    <t>Extintor</t>
-  </si>
-  <si>
-    <t>Moquetas</t>
-  </si>
-  <si>
-    <t>Tuercas Seguridad</t>
-  </si>
-  <si>
-    <t>Antena</t>
-  </si>
-  <si>
-    <t>Radio</t>
-  </si>
-  <si>
-    <t>Caja</t>
-  </si>
-  <si>
-    <t>Mica</t>
-  </si>
-  <si>
-    <t>Funda protectora</t>
-  </si>
-  <si>
-    <t>Cargador</t>
-  </si>
-  <si>
     <t>Codigo</t>
   </si>
   <si>
     <t>EFECTIVO</t>
   </si>
   <si>
-    <t>Efectivo</t>
-  </si>
-  <si>
     <t>TRANSFERENCIA</t>
   </si>
   <si>
-    <t>Transferencia</t>
-  </si>
-  <si>
     <t>TARJETA_CREDITO</t>
   </si>
   <si>
-    <t>Tarjeta de Credito</t>
-  </si>
-  <si>
     <t>TARJETA_DEBITO</t>
   </si>
   <si>
-    <t>Tarjeta de Debito</t>
-  </si>
-  <si>
     <t>MIXTA</t>
   </si>
   <si>
-    <t>Mixta</t>
-  </si>
-  <si>
     <t>OTRO</t>
   </si>
   <si>
-    <t>Otro</t>
-  </si>
-  <si>
     <t>Marca</t>
   </si>
   <si>
-    <t>Bosch</t>
-  </si>
-  <si>
-    <t>Denso</t>
-  </si>
-  <si>
     <t>NGK</t>
   </si>
   <si>
-    <t>Monroe</t>
-  </si>
-  <si>
     <t>KYB</t>
   </si>
   <si>
-    <t>Gates</t>
-  </si>
-  <si>
     <t>SKF</t>
   </si>
   <si>
-    <t>Valeo</t>
-  </si>
-  <si>
-    <t>Hella</t>
-  </si>
-  <si>
-    <t>Brembo</t>
-  </si>
-  <si>
     <t>TRW</t>
   </si>
   <si>
-    <t>Dayco</t>
-  </si>
-  <si>
-    <t>Continental</t>
-  </si>
-  <si>
-    <t>Mann-Filter</t>
-  </si>
-  <si>
-    <t>Mahle</t>
-  </si>
-  <si>
-    <t>ACDelco</t>
-  </si>
-  <si>
-    <t>Motorcraft</t>
-  </si>
-  <si>
-    <t>Mopar</t>
-  </si>
-  <si>
-    <t>Delphi</t>
-  </si>
-  <si>
-    <t>Aisin</t>
-  </si>
-  <si>
     <t>NTN</t>
   </si>
   <si>
-    <t>Koyo</t>
-  </si>
-  <si>
-    <t>Timken</t>
-  </si>
-  <si>
-    <t>Wagner</t>
-  </si>
-  <si>
-    <t>Champion</t>
-  </si>
-  <si>
-    <t>Febi Bilstein</t>
-  </si>
-  <si>
-    <t>Sachs</t>
-  </si>
-  <si>
-    <t>LuK</t>
-  </si>
-  <si>
     <t>INA</t>
   </si>
   <si>
-    <t>Fram</t>
-  </si>
-  <si>
-    <t>Wix</t>
-  </si>
-  <si>
-    <t>Castrol</t>
-  </si>
-  <si>
-    <t>Mobil</t>
-  </si>
-  <si>
-    <t>Shell</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
     <t>Motivo</t>
   </si>
   <si>
@@ -811,6 +544,264 @@
   </si>
   <si>
     <t>NIVEL BAJO DE LIQUIDO DE DIRECCION</t>
+  </si>
+  <si>
+    <t>SEDAN</t>
+  </si>
+  <si>
+    <t>CAMIONETA</t>
+  </si>
+  <si>
+    <t>JEEP</t>
+  </si>
+  <si>
+    <t>4X4</t>
+  </si>
+  <si>
+    <t>CAMION</t>
+  </si>
+  <si>
+    <t>HIBRIDO</t>
+  </si>
+  <si>
+    <t>ELECTRICO</t>
+  </si>
+  <si>
+    <t>CUPE</t>
+  </si>
+  <si>
+    <t>DOBLE CABINA</t>
+  </si>
+  <si>
+    <t>ROJO</t>
+  </si>
+  <si>
+    <t>AZUL</t>
+  </si>
+  <si>
+    <t>AMARILLO</t>
+  </si>
+  <si>
+    <t>VERDE</t>
+  </si>
+  <si>
+    <t>NARANJA</t>
+  </si>
+  <si>
+    <t>MORADO</t>
+  </si>
+  <si>
+    <t>ROSA</t>
+  </si>
+  <si>
+    <t>MARRON</t>
+  </si>
+  <si>
+    <t>BLANCO</t>
+  </si>
+  <si>
+    <t>NEGRO</t>
+  </si>
+  <si>
+    <t>GRIS</t>
+  </si>
+  <si>
+    <t>BEIGE</t>
+  </si>
+  <si>
+    <t>CREMA</t>
+  </si>
+  <si>
+    <t>MARFIL</t>
+  </si>
+  <si>
+    <t>CELESTE</t>
+  </si>
+  <si>
+    <t>AZUL OSCURO</t>
+  </si>
+  <si>
+    <t>VERDE CLARO</t>
+  </si>
+  <si>
+    <t>VERDE OSCURO</t>
+  </si>
+  <si>
+    <t>TURQUESA</t>
+  </si>
+  <si>
+    <t>CIAN</t>
+  </si>
+  <si>
+    <t>MAGENTA</t>
+  </si>
+  <si>
+    <t>VIOLETA</t>
+  </si>
+  <si>
+    <t>DORADO</t>
+  </si>
+  <si>
+    <t>PLATEADO</t>
+  </si>
+  <si>
+    <t>AZUL MARINO</t>
+  </si>
+  <si>
+    <t>LIMA</t>
+  </si>
+  <si>
+    <t>OLIVA</t>
+  </si>
+  <si>
+    <t>PLOMO</t>
+  </si>
+  <si>
+    <t>VINO</t>
+  </si>
+  <si>
+    <t>BRONCE</t>
+  </si>
+  <si>
+    <t>PERLA</t>
+  </si>
+  <si>
+    <t>CHAMPAGNE</t>
+  </si>
+  <si>
+    <t>HERRAMIENTAS VARIAS</t>
+  </si>
+  <si>
+    <t>GATA</t>
+  </si>
+  <si>
+    <t>TRIANGULO DE SEGURIDAD</t>
+  </si>
+  <si>
+    <t>BOTIQUIN</t>
+  </si>
+  <si>
+    <t>EXTINTOR</t>
+  </si>
+  <si>
+    <t>MOQUETAS</t>
+  </si>
+  <si>
+    <t>TUERCAS SEGURIDAD</t>
+  </si>
+  <si>
+    <t>ANTENA</t>
+  </si>
+  <si>
+    <t>RADIO</t>
+  </si>
+  <si>
+    <t>CAJA</t>
+  </si>
+  <si>
+    <t>MICA</t>
+  </si>
+  <si>
+    <t>FUNDA PROTECTORA</t>
+  </si>
+  <si>
+    <t>CARGADOR</t>
+  </si>
+  <si>
+    <t>TARJETA DE CREDITO</t>
+  </si>
+  <si>
+    <t>TARJETA DE DEBITO</t>
+  </si>
+  <si>
+    <t>BOSCH</t>
+  </si>
+  <si>
+    <t>DENSO</t>
+  </si>
+  <si>
+    <t>MONROE</t>
+  </si>
+  <si>
+    <t>GATES</t>
+  </si>
+  <si>
+    <t>VALEO</t>
+  </si>
+  <si>
+    <t>HELLA</t>
+  </si>
+  <si>
+    <t>BREMBO</t>
+  </si>
+  <si>
+    <t>DAYCO</t>
+  </si>
+  <si>
+    <t>CONTINENTAL</t>
+  </si>
+  <si>
+    <t>MANN-FILTER</t>
+  </si>
+  <si>
+    <t>MAHLE</t>
+  </si>
+  <si>
+    <t>ACDELCO</t>
+  </si>
+  <si>
+    <t>MOTORCRAFT</t>
+  </si>
+  <si>
+    <t>MOPAR</t>
+  </si>
+  <si>
+    <t>DELPHI</t>
+  </si>
+  <si>
+    <t>AISIN</t>
+  </si>
+  <si>
+    <t>KOYO</t>
+  </si>
+  <si>
+    <t>TIMKEN</t>
+  </si>
+  <si>
+    <t>WAGNER</t>
+  </si>
+  <si>
+    <t>CHAMPION</t>
+  </si>
+  <si>
+    <t>FEBI BILSTEIN</t>
+  </si>
+  <si>
+    <t>SACHS</t>
+  </si>
+  <si>
+    <t>LUK</t>
+  </si>
+  <si>
+    <t>FRAM</t>
+  </si>
+  <si>
+    <t>WIX</t>
+  </si>
+  <si>
+    <t>CASTROL</t>
+  </si>
+  <si>
+    <t>MOBIL</t>
+  </si>
+  <si>
+    <t>SHELL</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>GENERICA</t>
   </si>
 </sst>
 </file>
@@ -818,7 +809,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_ &quot;$&quot;* #,##0.00_ ;_ &quot;$&quot;* \-#,##0.00_ ;_ &quot;$&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ &quot;$&quot;* #,##0.00_ ;_ &quot;$&quot;* \-#,##0.00_ ;_ &quot;$&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -879,20 +870,20 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1191,10 +1182,32 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{09F135B8-0859-4C64-8A41-1C3785886324}">
+  <we:reference id="wa200009404" version="1.0.0.5" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.5" store="wa200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
@@ -1280,7 +1293,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
   </cols>
@@ -1292,57 +1305,57 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -1353,174 +1366,174 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>90</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>92</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>94</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>95</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>96</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>98</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>99</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>100</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>101</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>102</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>104</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>105</v>
+        <v>198</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>106</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>107</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>108</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>109</v>
+        <v>202</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>110</v>
+        <v>203</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>111</v>
+        <v>204</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>112</v>
+        <v>205</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>113</v>
+        <v>206</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>114</v>
+        <v>207</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>115</v>
+        <v>208</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>116</v>
+        <v>209</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>117</v>
+        <v>210</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>118</v>
+        <v>211</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>119</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -1531,79 +1544,79 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>121</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>122</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>125</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>126</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>127</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>128</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>129</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>130</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>131</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>132</v>
+        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -1614,7 +1627,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -1622,7 +1635,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>59</v>
@@ -1630,50 +1643,50 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>135</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>139</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>140</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>141</v>
+        <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>143</v>
+        <v>85</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>145</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
-        <v>146</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1683,190 +1696,195 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:A36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A37"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>152</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>153</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>155</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>156</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>158</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>159</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>160</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>161</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>162</v>
+        <v>238</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>163</v>
+        <v>239</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>164</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>165</v>
+        <v>241</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>166</v>
+        <v>242</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>167</v>
+        <v>243</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>168</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>169</v>
+        <v>244</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>170</v>
+        <v>245</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>171</v>
+        <v>246</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>172</v>
+        <v>247</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>173</v>
+        <v>248</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>174</v>
+        <v>249</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>175</v>
+        <v>250</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>176</v>
+        <v>93</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>177</v>
+        <v>251</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>178</v>
+        <v>252</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>179</v>
+        <v>253</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>180</v>
+        <v>254</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>181</v>
+        <v>255</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>182</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -1877,7 +1895,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
@@ -2398,24 +2416,24 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:A27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>183</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>184</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -2425,117 +2443,117 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>186</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>187</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>188</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>189</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>190</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>191</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>192</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>193</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>194</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>195</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>196</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>197</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>198</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>199</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>200</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>201</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>202</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>203</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>204</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>205</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>206</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>207</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>208</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2546,7 +2564,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:B55"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
@@ -2554,74 +2572,74 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>183</v>
+        <v>94</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>209</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>184</v>
+        <v>95</v>
       </c>
       <c r="B2" t="s">
-        <v>198</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>184</v>
+        <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>210</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>184</v>
+        <v>95</v>
       </c>
       <c r="B4" t="s">
-        <v>211</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>184</v>
+        <v>95</v>
       </c>
       <c r="B5" t="s">
-        <v>212</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>184</v>
+        <v>95</v>
       </c>
       <c r="B6" t="s">
-        <v>213</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>185</v>
+        <v>96</v>
       </c>
       <c r="B7" t="s">
-        <v>214</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>185</v>
+        <v>96</v>
       </c>
       <c r="B8" t="s">
-        <v>215</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>185</v>
+        <v>96</v>
       </c>
       <c r="B9" t="s">
-        <v>216</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -2637,7 +2655,7 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>217</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2645,7 +2663,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>218</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -2653,7 +2671,7 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>219</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -2661,335 +2679,335 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>220</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>186</v>
+        <v>97</v>
       </c>
       <c r="B15" t="s">
-        <v>221</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>186</v>
+        <v>97</v>
       </c>
       <c r="B16" t="s">
-        <v>222</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>186</v>
+        <v>97</v>
       </c>
       <c r="B17" t="s">
-        <v>223</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>186</v>
+        <v>97</v>
       </c>
       <c r="B18" t="s">
-        <v>224</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>187</v>
+        <v>98</v>
       </c>
       <c r="B19" t="s">
-        <v>225</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>187</v>
+        <v>98</v>
       </c>
       <c r="B20" t="s">
-        <v>226</v>
+        <v>137</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>187</v>
+        <v>98</v>
       </c>
       <c r="B21" t="s">
-        <v>227</v>
+        <v>138</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>187</v>
+        <v>98</v>
       </c>
       <c r="B22" t="s">
-        <v>228</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>188</v>
+        <v>99</v>
       </c>
       <c r="B23" t="s">
-        <v>229</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>188</v>
+        <v>99</v>
       </c>
       <c r="B24" t="s">
-        <v>230</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>188</v>
+        <v>99</v>
       </c>
       <c r="B25" t="s">
-        <v>231</v>
+        <v>142</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>188</v>
+        <v>99</v>
       </c>
       <c r="B26" t="s">
-        <v>232</v>
+        <v>143</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>189</v>
+        <v>100</v>
       </c>
       <c r="B27" t="s">
-        <v>233</v>
+        <v>144</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>189</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
-        <v>234</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>189</v>
+        <v>100</v>
       </c>
       <c r="B29" t="s">
-        <v>235</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>189</v>
+        <v>100</v>
       </c>
       <c r="B30" t="s">
-        <v>236</v>
+        <v>147</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>191</v>
+        <v>102</v>
       </c>
       <c r="B31" t="s">
-        <v>237</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>191</v>
+        <v>102</v>
       </c>
       <c r="B32" t="s">
-        <v>238</v>
+        <v>149</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>191</v>
+        <v>102</v>
       </c>
       <c r="B33" t="s">
-        <v>239</v>
+        <v>150</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>191</v>
+        <v>102</v>
       </c>
       <c r="B34" t="s">
-        <v>240</v>
+        <v>151</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>191</v>
+        <v>102</v>
       </c>
       <c r="B35" t="s">
-        <v>200</v>
+        <v>111</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>193</v>
+        <v>104</v>
       </c>
       <c r="B36" t="s">
-        <v>241</v>
+        <v>152</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>193</v>
+        <v>104</v>
       </c>
       <c r="B37" t="s">
-        <v>242</v>
+        <v>153</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>193</v>
+        <v>104</v>
       </c>
       <c r="B38" t="s">
-        <v>243</v>
+        <v>154</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>193</v>
+        <v>104</v>
       </c>
       <c r="B39" t="s">
-        <v>244</v>
+        <v>155</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>194</v>
+        <v>105</v>
       </c>
       <c r="B40" t="s">
-        <v>245</v>
+        <v>156</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>194</v>
+        <v>105</v>
       </c>
       <c r="B41" t="s">
-        <v>246</v>
+        <v>157</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>194</v>
+        <v>105</v>
       </c>
       <c r="B42" t="s">
-        <v>247</v>
+        <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>196</v>
+        <v>107</v>
       </c>
       <c r="B43" t="s">
-        <v>248</v>
+        <v>159</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>196</v>
+        <v>107</v>
       </c>
       <c r="B44" t="s">
-        <v>249</v>
+        <v>160</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>196</v>
+        <v>107</v>
       </c>
       <c r="B45" t="s">
-        <v>250</v>
+        <v>161</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>196</v>
+        <v>107</v>
       </c>
       <c r="B46" t="s">
-        <v>251</v>
+        <v>162</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>202</v>
+        <v>113</v>
       </c>
       <c r="B47" t="s">
-        <v>252</v>
+        <v>163</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>202</v>
+        <v>113</v>
       </c>
       <c r="B48" t="s">
-        <v>253</v>
+        <v>164</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>202</v>
+        <v>113</v>
       </c>
       <c r="B49" t="s">
-        <v>254</v>
+        <v>165</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>203</v>
+        <v>114</v>
       </c>
       <c r="B50" t="s">
-        <v>255</v>
+        <v>166</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>203</v>
+        <v>114</v>
       </c>
       <c r="B51" t="s">
-        <v>256</v>
+        <v>167</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>203</v>
+        <v>114</v>
       </c>
       <c r="B52" t="s">
-        <v>257</v>
+        <v>168</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>201</v>
+        <v>112</v>
       </c>
       <c r="B53" t="s">
-        <v>258</v>
+        <v>169</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>201</v>
+        <v>112</v>
       </c>
       <c r="B54" t="s">
-        <v>259</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>201</v>
+        <v>112</v>
       </c>
       <c r="B55" t="s">
-        <v>260</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add oil type catalog and capacity fields to vehicles, fix build errors
- New CatalogOilType entity with CRUD in DAO, repository, and settings UI
- Add oilType and oilCapacity fields to Vehicle entity with SearchableDropdown
- Database migration v7→v8, backup export/import support for oil types
- Add Aceites sheet to Catalogos.xlsx and generate_seed.py pipeline
- Fix typo in CustomerListScreen (oimport → import)
- Fix undefined isAdmin in WorkOrderDetailScreen by adding it to UiState

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Catalogos.xlsx
+++ b/data/Catalogos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rolan\AndroidStudioProjects\Serviaux\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38B21B18-45C6-48A9-A15A-D368C42949CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B4A8A6-6260-4280-BBDD-EC43EE8597D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usuarios" sheetId="1" r:id="rId1"/>
@@ -22,13 +22,377 @@
     <sheet name="Servicios" sheetId="7" r:id="rId7"/>
     <sheet name="Motivos" sheetId="8" r:id="rId8"/>
     <sheet name="Diagnosticos" sheetId="9" r:id="rId9"/>
+    <sheet name="Aceites" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="293">
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>Usuario</t>
+  </si>
+  <si>
+    <t>Rol</t>
+  </si>
+  <si>
+    <t>Contraseña</t>
+  </si>
+  <si>
+    <t>Andrés Sornoza</t>
+  </si>
+  <si>
+    <t>servielecar</t>
+  </si>
+  <si>
+    <t>ADMIN</t>
+  </si>
+  <si>
+    <t>f4d3s2a1</t>
+  </si>
+  <si>
+    <t>Nicole Plaza</t>
+  </si>
+  <si>
+    <t>nicopla</t>
+  </si>
+  <si>
+    <t>RECEPCIONISTA</t>
+  </si>
+  <si>
+    <t>Smith Mosquera</t>
+  </si>
+  <si>
+    <t>smimos</t>
+  </si>
+  <si>
+    <t>MECANICO</t>
+  </si>
+  <si>
+    <t>Ronny Mosquera</t>
+  </si>
+  <si>
+    <t>marciano</t>
+  </si>
+  <si>
+    <t>Tipo</t>
+  </si>
+  <si>
+    <t>SEDAN</t>
+  </si>
+  <si>
+    <t>SUV</t>
+  </si>
+  <si>
+    <t>CAMIONETA</t>
+  </si>
+  <si>
+    <t>JEEP</t>
+  </si>
+  <si>
+    <t>4X4</t>
+  </si>
+  <si>
+    <t>CAMION</t>
+  </si>
+  <si>
+    <t>HIBRIDO</t>
+  </si>
+  <si>
+    <t>ELECTRICO</t>
+  </si>
+  <si>
+    <t>CUPE</t>
+  </si>
+  <si>
+    <t>VAN</t>
+  </si>
+  <si>
+    <t>DOBLE CABINA</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>ROJO</t>
+  </si>
+  <si>
+    <t>AZUL</t>
+  </si>
+  <si>
+    <t>AMARILLO</t>
+  </si>
+  <si>
+    <t>VERDE</t>
+  </si>
+  <si>
+    <t>NARANJA</t>
+  </si>
+  <si>
+    <t>MORADO</t>
+  </si>
+  <si>
+    <t>ROSA</t>
+  </si>
+  <si>
+    <t>MARRON</t>
+  </si>
+  <si>
+    <t>BLANCO</t>
+  </si>
+  <si>
+    <t>NEGRO</t>
+  </si>
+  <si>
+    <t>GRIS</t>
+  </si>
+  <si>
+    <t>BEIGE</t>
+  </si>
+  <si>
+    <t>CREMA</t>
+  </si>
+  <si>
+    <t>MARFIL</t>
+  </si>
+  <si>
+    <t>CELESTE</t>
+  </si>
+  <si>
+    <t>AZUL OSCURO</t>
+  </si>
+  <si>
+    <t>VERDE CLARO</t>
+  </si>
+  <si>
+    <t>VERDE OSCURO</t>
+  </si>
+  <si>
+    <t>TURQUESA</t>
+  </si>
+  <si>
+    <t>CIAN</t>
+  </si>
+  <si>
+    <t>MAGENTA</t>
+  </si>
+  <si>
+    <t>VIOLETA</t>
+  </si>
+  <si>
+    <t>DORADO</t>
+  </si>
+  <si>
+    <t>PLATEADO</t>
+  </si>
+  <si>
+    <t>AZUL MARINO</t>
+  </si>
+  <si>
+    <t>LIMA</t>
+  </si>
+  <si>
+    <t>OLIVA</t>
+  </si>
+  <si>
+    <t>PLOMO</t>
+  </si>
+  <si>
+    <t>VINO</t>
+  </si>
+  <si>
+    <t>BRONCE</t>
+  </si>
+  <si>
+    <t>PERLA</t>
+  </si>
+  <si>
+    <t>CHAMPAGNE</t>
+  </si>
+  <si>
+    <t>Accesorio</t>
+  </si>
+  <si>
+    <t>HERRAMIENTAS VARIAS</t>
+  </si>
+  <si>
+    <t>GATA</t>
+  </si>
+  <si>
+    <t>TRIANGULO DE SEGURIDAD</t>
+  </si>
+  <si>
+    <t>BOTIQUIN</t>
+  </si>
+  <si>
+    <t>EXTINTOR</t>
+  </si>
+  <si>
+    <t>MOQUETAS</t>
+  </si>
+  <si>
+    <t>TUERCAS SEGURIDAD</t>
+  </si>
+  <si>
+    <t>ANTENA</t>
+  </si>
+  <si>
+    <t>RADIO</t>
+  </si>
+  <si>
+    <t>CAJA</t>
+  </si>
+  <si>
+    <t>MICA</t>
+  </si>
+  <si>
+    <t>FUNDA PROTECTORA</t>
+  </si>
+  <si>
+    <t>CARGADOR</t>
+  </si>
+  <si>
+    <t>Codigo</t>
+  </si>
+  <si>
+    <t>EFECTIVO</t>
+  </si>
+  <si>
+    <t>TRANSFERENCIA</t>
+  </si>
+  <si>
+    <t>TARJETA_CREDITO</t>
+  </si>
+  <si>
+    <t>TARJETA DE CREDITO</t>
+  </si>
+  <si>
+    <t>TARJETA_DEBITO</t>
+  </si>
+  <si>
+    <t>TARJETA DE DEBITO</t>
+  </si>
+  <si>
+    <t>MIXTA</t>
+  </si>
+  <si>
+    <t>OTRO</t>
+  </si>
+  <si>
+    <t>Marca</t>
+  </si>
+  <si>
+    <t>BOSCH</t>
+  </si>
+  <si>
+    <t>DENSO</t>
+  </si>
+  <si>
+    <t>NGK</t>
+  </si>
+  <si>
+    <t>MONROE</t>
+  </si>
+  <si>
+    <t>KYB</t>
+  </si>
+  <si>
+    <t>GATES</t>
+  </si>
+  <si>
+    <t>SKF</t>
+  </si>
+  <si>
+    <t>VALEO</t>
+  </si>
+  <si>
+    <t>HELLA</t>
+  </si>
+  <si>
+    <t>BREMBO</t>
+  </si>
+  <si>
+    <t>TRW</t>
+  </si>
+  <si>
+    <t>DAYCO</t>
+  </si>
+  <si>
+    <t>CONTINENTAL</t>
+  </si>
+  <si>
+    <t>MANN-FILTER</t>
+  </si>
+  <si>
+    <t>MAHLE</t>
+  </si>
+  <si>
+    <t>ACDELCO</t>
+  </si>
+  <si>
+    <t>MOTORCRAFT</t>
+  </si>
+  <si>
+    <t>MOPAR</t>
+  </si>
+  <si>
+    <t>DELPHI</t>
+  </si>
+  <si>
+    <t>AISIN</t>
+  </si>
+  <si>
+    <t>NTN</t>
+  </si>
+  <si>
+    <t>KOYO</t>
+  </si>
+  <si>
+    <t>TIMKEN</t>
+  </si>
+  <si>
+    <t>WAGNER</t>
+  </si>
+  <si>
+    <t>CHAMPION</t>
+  </si>
+  <si>
+    <t>FEBI BILSTEIN</t>
+  </si>
+  <si>
+    <t>SACHS</t>
+  </si>
+  <si>
+    <t>LUK</t>
+  </si>
+  <si>
+    <t>INA</t>
+  </si>
+  <si>
+    <t>FRAM</t>
+  </si>
+  <si>
+    <t>WIX</t>
+  </si>
+  <si>
+    <t>CASTROL</t>
+  </si>
+  <si>
+    <t>MOBIL</t>
+  </si>
+  <si>
+    <t>SHELL</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>GENERICA</t>
+  </si>
   <si>
     <t>Categoria</t>
   </si>
@@ -207,111 +571,6 @@
     <t>CAMBIOS MANGUERAS</t>
   </si>
   <si>
-    <t>Nombre</t>
-  </si>
-  <si>
-    <t>Usuario</t>
-  </si>
-  <si>
-    <t>Rol</t>
-  </si>
-  <si>
-    <t>Contraseña</t>
-  </si>
-  <si>
-    <t>Andrés Sornoza</t>
-  </si>
-  <si>
-    <t>servielecar</t>
-  </si>
-  <si>
-    <t>ADMIN</t>
-  </si>
-  <si>
-    <t>f4d3s2a1</t>
-  </si>
-  <si>
-    <t>Nicole Plaza</t>
-  </si>
-  <si>
-    <t>nicopla</t>
-  </si>
-  <si>
-    <t>RECEPCIONISTA</t>
-  </si>
-  <si>
-    <t>Smith Mosquera</t>
-  </si>
-  <si>
-    <t>smimos</t>
-  </si>
-  <si>
-    <t>MECANICO</t>
-  </si>
-  <si>
-    <t>Ronny Mosquera</t>
-  </si>
-  <si>
-    <t>marciano</t>
-  </si>
-  <si>
-    <t>Tipo</t>
-  </si>
-  <si>
-    <t>SUV</t>
-  </si>
-  <si>
-    <t>VAN</t>
-  </si>
-  <si>
-    <t>Color</t>
-  </si>
-  <si>
-    <t>Accesorio</t>
-  </si>
-  <si>
-    <t>Codigo</t>
-  </si>
-  <si>
-    <t>EFECTIVO</t>
-  </si>
-  <si>
-    <t>TRANSFERENCIA</t>
-  </si>
-  <si>
-    <t>TARJETA_CREDITO</t>
-  </si>
-  <si>
-    <t>TARJETA_DEBITO</t>
-  </si>
-  <si>
-    <t>MIXTA</t>
-  </si>
-  <si>
-    <t>OTRO</t>
-  </si>
-  <si>
-    <t>Marca</t>
-  </si>
-  <si>
-    <t>NGK</t>
-  </si>
-  <si>
-    <t>KYB</t>
-  </si>
-  <si>
-    <t>SKF</t>
-  </si>
-  <si>
-    <t>TRW</t>
-  </si>
-  <si>
-    <t>NTN</t>
-  </si>
-  <si>
-    <t>INA</t>
-  </si>
-  <si>
     <t>Motivo</t>
   </si>
   <si>
@@ -546,262 +805,109 @@
     <t>NIVEL BAJO DE LIQUIDO DE DIRECCION</t>
   </si>
   <si>
-    <t>SEDAN</t>
-  </si>
-  <si>
-    <t>CAMIONETA</t>
-  </si>
-  <si>
-    <t>JEEP</t>
-  </si>
-  <si>
-    <t>4X4</t>
-  </si>
-  <si>
-    <t>CAMION</t>
-  </si>
-  <si>
-    <t>HIBRIDO</t>
-  </si>
-  <si>
-    <t>ELECTRICO</t>
-  </si>
-  <si>
-    <t>CUPE</t>
-  </si>
-  <si>
-    <t>DOBLE CABINA</t>
-  </si>
-  <si>
-    <t>ROJO</t>
-  </si>
-  <si>
-    <t>AZUL</t>
-  </si>
-  <si>
-    <t>AMARILLO</t>
-  </si>
-  <si>
-    <t>VERDE</t>
-  </si>
-  <si>
-    <t>NARANJA</t>
-  </si>
-  <si>
-    <t>MORADO</t>
-  </si>
-  <si>
-    <t>ROSA</t>
-  </si>
-  <si>
-    <t>MARRON</t>
-  </si>
-  <si>
-    <t>BLANCO</t>
-  </si>
-  <si>
-    <t>NEGRO</t>
-  </si>
-  <si>
-    <t>GRIS</t>
-  </si>
-  <si>
-    <t>BEIGE</t>
-  </si>
-  <si>
-    <t>CREMA</t>
-  </si>
-  <si>
-    <t>MARFIL</t>
-  </si>
-  <si>
-    <t>CELESTE</t>
-  </si>
-  <si>
-    <t>AZUL OSCURO</t>
-  </si>
-  <si>
-    <t>VERDE CLARO</t>
-  </si>
-  <si>
-    <t>VERDE OSCURO</t>
-  </si>
-  <si>
-    <t>TURQUESA</t>
-  </si>
-  <si>
-    <t>CIAN</t>
-  </si>
-  <si>
-    <t>MAGENTA</t>
-  </si>
-  <si>
-    <t>VIOLETA</t>
-  </si>
-  <si>
-    <t>DORADO</t>
-  </si>
-  <si>
-    <t>PLATEADO</t>
-  </si>
-  <si>
-    <t>AZUL MARINO</t>
-  </si>
-  <si>
-    <t>LIMA</t>
-  </si>
-  <si>
-    <t>OLIVA</t>
-  </si>
-  <si>
-    <t>PLOMO</t>
-  </si>
-  <si>
-    <t>VINO</t>
-  </si>
-  <si>
-    <t>BRONCE</t>
-  </si>
-  <si>
-    <t>PERLA</t>
-  </si>
-  <si>
-    <t>CHAMPAGNE</t>
-  </si>
-  <si>
-    <t>HERRAMIENTAS VARIAS</t>
-  </si>
-  <si>
-    <t>GATA</t>
-  </si>
-  <si>
-    <t>TRIANGULO DE SEGURIDAD</t>
-  </si>
-  <si>
-    <t>BOTIQUIN</t>
-  </si>
-  <si>
-    <t>EXTINTOR</t>
-  </si>
-  <si>
-    <t>MOQUETAS</t>
-  </si>
-  <si>
-    <t>TUERCAS SEGURIDAD</t>
-  </si>
-  <si>
-    <t>ANTENA</t>
-  </si>
-  <si>
-    <t>RADIO</t>
-  </si>
-  <si>
-    <t>CAJA</t>
-  </si>
-  <si>
-    <t>MICA</t>
-  </si>
-  <si>
-    <t>FUNDA PROTECTORA</t>
-  </si>
-  <si>
-    <t>CARGADOR</t>
-  </si>
-  <si>
-    <t>TARJETA DE CREDITO</t>
-  </si>
-  <si>
-    <t>TARJETA DE DEBITO</t>
-  </si>
-  <si>
-    <t>BOSCH</t>
-  </si>
-  <si>
-    <t>DENSO</t>
-  </si>
-  <si>
-    <t>MONROE</t>
-  </si>
-  <si>
-    <t>GATES</t>
-  </si>
-  <si>
-    <t>VALEO</t>
-  </si>
-  <si>
-    <t>HELLA</t>
-  </si>
-  <si>
-    <t>BREMBO</t>
-  </si>
-  <si>
-    <t>DAYCO</t>
-  </si>
-  <si>
-    <t>CONTINENTAL</t>
-  </si>
-  <si>
-    <t>MANN-FILTER</t>
-  </si>
-  <si>
-    <t>MAHLE</t>
-  </si>
-  <si>
-    <t>ACDELCO</t>
-  </si>
-  <si>
-    <t>MOTORCRAFT</t>
-  </si>
-  <si>
-    <t>MOPAR</t>
-  </si>
-  <si>
-    <t>DELPHI</t>
-  </si>
-  <si>
-    <t>AISIN</t>
-  </si>
-  <si>
-    <t>KOYO</t>
-  </si>
-  <si>
-    <t>TIMKEN</t>
-  </si>
-  <si>
-    <t>WAGNER</t>
-  </si>
-  <si>
-    <t>CHAMPION</t>
-  </si>
-  <si>
-    <t>FEBI BILSTEIN</t>
-  </si>
-  <si>
-    <t>SACHS</t>
-  </si>
-  <si>
-    <t>LUK</t>
-  </si>
-  <si>
-    <t>FRAM</t>
-  </si>
-  <si>
-    <t>WIX</t>
-  </si>
-  <si>
-    <t>CASTROL</t>
-  </si>
-  <si>
-    <t>MOBIL</t>
-  </si>
-  <si>
-    <t>SHELL</t>
-  </si>
-  <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>GENERICA</t>
+    <t>Tipo de Aceite</t>
+  </si>
+  <si>
+    <t>0W-16</t>
+  </si>
+  <si>
+    <t>0W-20</t>
+  </si>
+  <si>
+    <t>0W-30</t>
+  </si>
+  <si>
+    <t>0W-40</t>
+  </si>
+  <si>
+    <t>5W-20</t>
+  </si>
+  <si>
+    <t>5W-30</t>
+  </si>
+  <si>
+    <t>5W-40</t>
+  </si>
+  <si>
+    <t>5W-50</t>
+  </si>
+  <si>
+    <t>10W-30</t>
+  </si>
+  <si>
+    <t>10W-40</t>
+  </si>
+  <si>
+    <t>10W-50</t>
+  </si>
+  <si>
+    <t>10W-60</t>
+  </si>
+  <si>
+    <t>15W-40</t>
+  </si>
+  <si>
+    <t>15W-50</t>
+  </si>
+  <si>
+    <t>20W-50</t>
+  </si>
+  <si>
+    <t>20W-60</t>
+  </si>
+  <si>
+    <t>25W-50</t>
+  </si>
+  <si>
+    <t>25W-60</t>
+  </si>
+  <si>
+    <t>SAE 30</t>
+  </si>
+  <si>
+    <t>SAE 40</t>
+  </si>
+  <si>
+    <t>SAE 50</t>
+  </si>
+  <si>
+    <t>ATF</t>
+  </si>
+  <si>
+    <t>ATF+4</t>
+  </si>
+  <si>
+    <t>ATF DEXRON III</t>
+  </si>
+  <si>
+    <t>ATF DEXRON VI</t>
+  </si>
+  <si>
+    <t>CVT</t>
+  </si>
+  <si>
+    <t>DCT</t>
+  </si>
+  <si>
+    <t>75W-80</t>
+  </si>
+  <si>
+    <t>75W-85</t>
+  </si>
+  <si>
+    <t>75W-90</t>
+  </si>
+  <si>
+    <t>75W-140</t>
+  </si>
+  <si>
+    <t>80W-90</t>
+  </si>
+  <si>
+    <t>85W-140</t>
+  </si>
+  <si>
+    <t>ACEITE 2 TIEMPOS</t>
   </si>
 </sst>
 </file>
@@ -1182,28 +1288,6 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="1">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{09F135B8-0859-4C64-8A41-1C3785886324}">
-  <we:reference id="wa200009404" version="1.0.0.5" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="wa200009404" version="1.0.0.5" store="wa200009404" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D5"/>
@@ -1217,72 +1301,257 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>61</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>62</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>66</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>66</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:A35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -1300,62 +1569,62 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>173</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>174</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>175</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>176</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>177</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>178</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>179</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>180</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1373,167 +1642,167 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>181</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>182</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>183</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>184</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>185</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>187</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>188</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>189</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>190</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>191</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>192</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>193</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>194</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>195</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>196</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>197</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>198</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>199</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>200</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>201</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>202</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>203</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>204</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>205</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>206</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>207</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>208</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>209</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>210</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>211</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>212</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1551,72 +1820,72 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>213</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>214</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>215</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>216</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>217</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>218</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>219</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>220</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>221</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>222</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>223</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>224</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>225</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1635,58 +1904,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B4" t="s">
-        <v>226</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B5" t="s">
-        <v>227</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1704,27 +1973,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>228</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>229</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>230</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
@@ -1734,157 +2003,157 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>231</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>232</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>233</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>234</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>235</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>236</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>237</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>238</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>239</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>240</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>241</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>242</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>243</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>244</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>245</v>
+        <v>107</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>246</v>
+        <v>108</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>247</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>248</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>249</v>
+        <v>111</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>250</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>251</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>252</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>253</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>254</v>
+        <v>117</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>255</v>
+        <v>118</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>256</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>257</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1904,21 +2173,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>122</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>125</v>
       </c>
       <c r="C2" s="2">
         <v>5</v>
@@ -1926,10 +2195,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>126</v>
       </c>
       <c r="C3" s="2">
         <v>5</v>
@@ -1937,10 +2206,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>127</v>
       </c>
       <c r="C4" s="2">
         <v>20</v>
@@ -1948,10 +2217,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>128</v>
       </c>
       <c r="C5" s="2">
         <v>10</v>
@@ -1959,10 +2228,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>129</v>
       </c>
       <c r="C6" s="2">
         <v>60</v>
@@ -1970,10 +2239,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>130</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>131</v>
       </c>
       <c r="C7" s="2">
         <v>15</v>
@@ -1981,10 +2250,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>130</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>132</v>
       </c>
       <c r="C8" s="2">
         <v>25</v>
@@ -1992,10 +2261,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>130</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>133</v>
       </c>
       <c r="C9" s="2">
         <v>20</v>
@@ -2003,10 +2272,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>130</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>134</v>
       </c>
       <c r="C10" s="2">
         <v>40</v>
@@ -2014,10 +2283,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>130</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>135</v>
       </c>
       <c r="C11" s="2">
         <v>50</v>
@@ -2025,10 +2294,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>130</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>136</v>
       </c>
       <c r="C12" s="2">
         <v>30</v>
@@ -2036,10 +2305,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>137</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>138</v>
       </c>
       <c r="C13" s="2">
         <v>300</v>
@@ -2047,10 +2316,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>137</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>139</v>
       </c>
       <c r="C14" s="2">
         <v>450</v>
@@ -2058,10 +2327,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>140</v>
       </c>
       <c r="B15" t="s">
-        <v>20</v>
+        <v>141</v>
       </c>
       <c r="C15" s="2">
         <v>60</v>
@@ -2069,10 +2338,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>140</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>142</v>
       </c>
       <c r="C16" s="2">
         <v>50</v>
@@ -2080,10 +2349,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>144</v>
       </c>
       <c r="C17" s="2">
         <v>30</v>
@@ -2091,10 +2360,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>145</v>
       </c>
       <c r="C18" s="2">
         <v>30</v>
@@ -2102,10 +2371,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>146</v>
       </c>
       <c r="C19" s="2">
         <v>15</v>
@@ -2113,10 +2382,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="C20" s="2">
         <v>15</v>
@@ -2124,10 +2393,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>148</v>
       </c>
       <c r="C21" s="2">
         <v>20</v>
@@ -2135,10 +2404,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
       <c r="B22" t="s">
-        <v>29</v>
+        <v>150</v>
       </c>
       <c r="C22" s="2">
         <v>10</v>
@@ -2146,10 +2415,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
       <c r="B23" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="C23" s="2">
         <v>30</v>
@@ -2157,10 +2426,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>152</v>
       </c>
       <c r="C24" s="2">
         <v>100</v>
@@ -2168,10 +2437,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>153</v>
       </c>
       <c r="C25" s="2">
         <v>100</v>
@@ -2179,10 +2448,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
       <c r="B26" t="s">
-        <v>33</v>
+        <v>154</v>
       </c>
       <c r="C26" s="2">
         <v>20</v>
@@ -2190,10 +2459,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
       <c r="B27" t="s">
-        <v>34</v>
+        <v>155</v>
       </c>
       <c r="C27" s="2">
         <v>20</v>
@@ -2201,10 +2470,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
       <c r="B28" t="s">
-        <v>35</v>
+        <v>156</v>
       </c>
       <c r="C28" s="2">
         <v>80</v>
@@ -2212,10 +2481,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>157</v>
       </c>
       <c r="C29" s="2">
         <v>50</v>
@@ -2223,10 +2492,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>158</v>
       </c>
       <c r="B30" t="s">
-        <v>38</v>
+        <v>159</v>
       </c>
       <c r="C30" s="2">
         <v>60</v>
@@ -2234,10 +2503,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>158</v>
       </c>
       <c r="B31" t="s">
-        <v>39</v>
+        <v>160</v>
       </c>
       <c r="C31" s="2">
         <v>30</v>
@@ -2245,10 +2514,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>158</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>161</v>
       </c>
       <c r="C32" s="2">
         <v>60</v>
@@ -2256,10 +2525,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>158</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>162</v>
       </c>
       <c r="C33" s="2">
         <v>80</v>
@@ -2267,10 +2536,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>42</v>
+        <v>163</v>
       </c>
       <c r="B34" t="s">
-        <v>43</v>
+        <v>164</v>
       </c>
       <c r="C34" s="2">
         <v>5</v>
@@ -2278,10 +2547,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>42</v>
+        <v>163</v>
       </c>
       <c r="B35" t="s">
-        <v>44</v>
+        <v>165</v>
       </c>
       <c r="C35" s="2">
         <v>10</v>
@@ -2289,10 +2558,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>42</v>
+        <v>163</v>
       </c>
       <c r="B36" t="s">
-        <v>45</v>
+        <v>166</v>
       </c>
       <c r="C36" s="2">
         <v>10</v>
@@ -2300,10 +2569,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>42</v>
+        <v>163</v>
       </c>
       <c r="B37" t="s">
-        <v>46</v>
+        <v>167</v>
       </c>
       <c r="C37" s="2">
         <v>30</v>
@@ -2311,10 +2580,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>42</v>
+        <v>163</v>
       </c>
       <c r="B38" t="s">
-        <v>47</v>
+        <v>168</v>
       </c>
       <c r="C38" s="2">
         <v>40</v>
@@ -2322,10 +2591,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>42</v>
+        <v>163</v>
       </c>
       <c r="B39" t="s">
-        <v>48</v>
+        <v>169</v>
       </c>
       <c r="C39" s="2">
         <v>5</v>
@@ -2333,10 +2602,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>49</v>
+        <v>170</v>
       </c>
       <c r="B40" t="s">
-        <v>50</v>
+        <v>171</v>
       </c>
       <c r="C40" s="2">
         <v>70</v>
@@ -2344,10 +2613,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>51</v>
+        <v>172</v>
       </c>
       <c r="B41" t="s">
-        <v>52</v>
+        <v>173</v>
       </c>
       <c r="C41" s="2">
         <v>10</v>
@@ -2355,10 +2624,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>172</v>
       </c>
       <c r="B42" t="s">
-        <v>53</v>
+        <v>174</v>
       </c>
       <c r="C42" s="2">
         <v>15</v>
@@ -2366,10 +2635,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>51</v>
+        <v>172</v>
       </c>
       <c r="B43" t="s">
-        <v>54</v>
+        <v>175</v>
       </c>
       <c r="C43" s="2">
         <v>50</v>
@@ -2377,10 +2646,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>55</v>
+        <v>176</v>
       </c>
       <c r="B44" t="s">
-        <v>56</v>
+        <v>177</v>
       </c>
       <c r="C44" s="2">
         <v>10</v>
@@ -2388,10 +2657,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>55</v>
+        <v>176</v>
       </c>
       <c r="B45" t="s">
-        <v>57</v>
+        <v>178</v>
       </c>
       <c r="C45" s="2">
         <v>20</v>
@@ -2399,10 +2668,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>55</v>
+        <v>176</v>
       </c>
       <c r="B46" t="s">
-        <v>58</v>
+        <v>179</v>
       </c>
       <c r="C46" s="2">
         <v>10</v>
@@ -2423,137 +2692,137 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>94</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>98</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>102</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>103</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>104</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>105</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>106</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>107</v>
+        <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>108</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>109</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>110</v>
+        <v>196</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>111</v>
+        <v>197</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>112</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>113</v>
+        <v>199</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>114</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>115</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>116</v>
+        <v>202</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>117</v>
+        <v>203</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>118</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>119</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2572,442 +2841,442 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>94</v>
+        <v>180</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>120</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>181</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>181</v>
       </c>
       <c r="B3" t="s">
-        <v>121</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>95</v>
+        <v>181</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>181</v>
       </c>
       <c r="B5" t="s">
-        <v>123</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>181</v>
       </c>
       <c r="B6" t="s">
-        <v>124</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>96</v>
+        <v>182</v>
       </c>
       <c r="B7" t="s">
-        <v>125</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>182</v>
       </c>
       <c r="B8" t="s">
-        <v>126</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>96</v>
+        <v>182</v>
       </c>
       <c r="B9" t="s">
-        <v>127</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B10" t="s">
-        <v>4</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B11" t="s">
-        <v>128</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B12" t="s">
-        <v>129</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B13" t="s">
-        <v>130</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="B14" t="s">
-        <v>131</v>
+        <v>217</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>97</v>
+        <v>183</v>
       </c>
       <c r="B15" t="s">
-        <v>132</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>183</v>
       </c>
       <c r="B16" t="s">
-        <v>133</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>97</v>
+        <v>183</v>
       </c>
       <c r="B17" t="s">
-        <v>134</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>97</v>
+        <v>183</v>
       </c>
       <c r="B18" t="s">
-        <v>135</v>
+        <v>221</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>184</v>
       </c>
       <c r="B19" t="s">
-        <v>136</v>
+        <v>222</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>98</v>
+        <v>184</v>
       </c>
       <c r="B20" t="s">
-        <v>137</v>
+        <v>223</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>98</v>
+        <v>184</v>
       </c>
       <c r="B21" t="s">
-        <v>138</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>184</v>
       </c>
       <c r="B22" t="s">
-        <v>139</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>99</v>
+        <v>185</v>
       </c>
       <c r="B23" t="s">
-        <v>140</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>99</v>
+        <v>185</v>
       </c>
       <c r="B24" t="s">
-        <v>141</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>99</v>
+        <v>185</v>
       </c>
       <c r="B25" t="s">
-        <v>142</v>
+        <v>228</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>99</v>
+        <v>185</v>
       </c>
       <c r="B26" t="s">
-        <v>143</v>
+        <v>229</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>100</v>
+        <v>186</v>
       </c>
       <c r="B27" t="s">
-        <v>144</v>
+        <v>230</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>100</v>
+        <v>186</v>
       </c>
       <c r="B28" t="s">
-        <v>145</v>
+        <v>231</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>100</v>
+        <v>186</v>
       </c>
       <c r="B29" t="s">
-        <v>146</v>
+        <v>232</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>100</v>
+        <v>186</v>
       </c>
       <c r="B30" t="s">
-        <v>147</v>
+        <v>233</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>102</v>
+        <v>188</v>
       </c>
       <c r="B31" t="s">
-        <v>148</v>
+        <v>234</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>102</v>
+        <v>188</v>
       </c>
       <c r="B32" t="s">
-        <v>149</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>102</v>
+        <v>188</v>
       </c>
       <c r="B33" t="s">
-        <v>150</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>102</v>
+        <v>188</v>
       </c>
       <c r="B34" t="s">
-        <v>151</v>
+        <v>237</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>102</v>
+        <v>188</v>
       </c>
       <c r="B35" t="s">
-        <v>111</v>
+        <v>197</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>104</v>
+        <v>190</v>
       </c>
       <c r="B36" t="s">
-        <v>152</v>
+        <v>238</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>104</v>
+        <v>190</v>
       </c>
       <c r="B37" t="s">
-        <v>153</v>
+        <v>239</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>104</v>
+        <v>190</v>
       </c>
       <c r="B38" t="s">
-        <v>154</v>
+        <v>240</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>104</v>
+        <v>190</v>
       </c>
       <c r="B39" t="s">
-        <v>155</v>
+        <v>241</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>105</v>
+        <v>191</v>
       </c>
       <c r="B40" t="s">
-        <v>156</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>105</v>
+        <v>191</v>
       </c>
       <c r="B41" t="s">
-        <v>157</v>
+        <v>243</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>105</v>
+        <v>191</v>
       </c>
       <c r="B42" t="s">
-        <v>158</v>
+        <v>244</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>107</v>
+        <v>193</v>
       </c>
       <c r="B43" t="s">
-        <v>159</v>
+        <v>245</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>107</v>
+        <v>193</v>
       </c>
       <c r="B44" t="s">
-        <v>160</v>
+        <v>246</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>107</v>
+        <v>193</v>
       </c>
       <c r="B45" t="s">
-        <v>161</v>
+        <v>247</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>107</v>
+        <v>193</v>
       </c>
       <c r="B46" t="s">
-        <v>162</v>
+        <v>248</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>113</v>
+        <v>199</v>
       </c>
       <c r="B47" t="s">
-        <v>163</v>
+        <v>249</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>113</v>
+        <v>199</v>
       </c>
       <c r="B48" t="s">
-        <v>164</v>
+        <v>250</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>113</v>
+        <v>199</v>
       </c>
       <c r="B49" t="s">
-        <v>165</v>
+        <v>251</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>114</v>
+        <v>200</v>
       </c>
       <c r="B50" t="s">
-        <v>166</v>
+        <v>252</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>114</v>
+        <v>200</v>
       </c>
       <c r="B51" t="s">
-        <v>167</v>
+        <v>253</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>114</v>
+        <v>200</v>
       </c>
       <c r="B52" t="s">
-        <v>168</v>
+        <v>254</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>112</v>
+        <v>198</v>
       </c>
       <c r="B53" t="s">
-        <v>169</v>
+        <v>255</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>112</v>
+        <v>198</v>
       </c>
       <c r="B54" t="s">
-        <v>170</v>
+        <v>256</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>112</v>
+        <v>198</v>
       </c>
       <c r="B55" t="s">
-        <v>171</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add appointment system, admission date, and reset DB to version 1
- Implement full appointment (turnos) system: entity, DAO, repository,
  ViewModel, list/form screens with status filtering and CRUD
- Add appointment-to-work-order conversion flow with prefilled fields
- Add admissionDate field to WorkOrder (separate from automatic createdAt)
- Add Turnos tab to bottom navigation bar
- Update dashboard with appointment counters
- Update backup/restore to include appointments
- Remove all database migrations and reset to version 1 (clean schema)
- Rename DB from "serviaux_v1" to "serviaux" with destructive fallback
- Update generate_seed.py to read commission columns from Excel

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Catalogos.xlsx
+++ b/data/Catalogos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rolan\AndroidStudioProjects\Serviaux\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B4A8A6-6260-4280-BBDD-EC43EE8597D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AACC40-FD26-4ADF-BC56-7168AA168872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usuarios" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="297">
   <si>
     <t>Nombre</t>
   </si>
@@ -908,6 +908,18 @@
   </si>
   <si>
     <t>ACEITE 2 TIEMPOS</t>
+  </si>
+  <si>
+    <t>Comisiona</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>ValorComision</t>
   </si>
 </sst>
 </file>
@@ -1290,16 +1302,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="3" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1310,10 +1322,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1323,11 +1341,11 @@
       <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1337,11 +1355,11 @@
       <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1352,10 +1370,16 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
+        <v>294</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1366,6 +1390,12 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
+        <v>295</v>
+      </c>
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>